<commit_message>
add time computattion, resolve financial statments in share Rmd, add try catch in ecb bond fetching
</commit_message>
<xml_diff>
--- a/data/excel/kof_barometer_swiss.xlsx
+++ b/data/excel/kof_barometer_swiss.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B424"/>
+  <dimension ref="A1:B425"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -390,7 +390,7 @@
         <v>1991-01</v>
       </c>
       <c r="B2">
-        <v>87.8117481093321</v>
+        <v>87.8134683637333</v>
       </c>
     </row>
     <row r="3">
@@ -398,7 +398,7 @@
         <v>1991-02</v>
       </c>
       <c r="B3">
-        <v>78.3174438576769</v>
+        <v>78.3206605849094</v>
       </c>
     </row>
     <row r="4">
@@ -406,7 +406,7 @@
         <v>1991-03</v>
       </c>
       <c r="B4">
-        <v>85.1824477315286</v>
+        <v>85.1845824108815</v>
       </c>
     </row>
     <row r="5">
@@ -414,7 +414,7 @@
         <v>1991-04</v>
       </c>
       <c r="B5">
-        <v>91.8159821295335</v>
+        <v>91.8170712447525</v>
       </c>
     </row>
     <row r="6">
@@ -422,7 +422,7 @@
         <v>1991-05</v>
       </c>
       <c r="B6">
-        <v>90.3307950834112</v>
+        <v>90.3321182907769</v>
       </c>
     </row>
     <row r="7">
@@ -430,7 +430,7 @@
         <v>1991-06</v>
       </c>
       <c r="B7">
-        <v>89.2677889927382</v>
+        <v>89.2692797489513</v>
       </c>
     </row>
     <row r="8">
@@ -438,7 +438,7 @@
         <v>1991-07</v>
       </c>
       <c r="B8">
-        <v>92.0093832203799</v>
+        <v>92.0104418521143</v>
       </c>
     </row>
     <row r="9">
@@ -446,7 +446,7 @@
         <v>1991-08</v>
       </c>
       <c r="B9">
-        <v>98.5784858412557</v>
+        <v>98.5785090644612</v>
       </c>
     </row>
     <row r="10">
@@ -454,7 +454,7 @@
         <v>1991-09</v>
       </c>
       <c r="B10">
-        <v>102.53201654656</v>
+        <v>102.531416622337</v>
       </c>
     </row>
     <row r="11">
@@ -462,7 +462,7 @@
         <v>1991-10</v>
       </c>
       <c r="B11">
-        <v>102.069496051354</v>
+        <v>102.068969028665</v>
       </c>
     </row>
     <row r="12">
@@ -470,7 +470,7 @@
         <v>1991-11</v>
       </c>
       <c r="B12">
-        <v>100.080079777192</v>
+        <v>100.07986632223</v>
       </c>
     </row>
     <row r="13">
@@ -478,7 +478,7 @@
         <v>1991-12</v>
       </c>
       <c r="B13">
-        <v>100.794590789097</v>
+        <v>100.79426471437</v>
       </c>
     </row>
     <row r="14">
@@ -486,7 +486,7 @@
         <v>1992-01</v>
       </c>
       <c r="B14">
-        <v>101.026644597417</v>
+        <v>101.026281946843</v>
       </c>
     </row>
     <row r="15">
@@ -494,7 +494,7 @@
         <v>1992-02</v>
       </c>
       <c r="B15">
-        <v>105.582720846927</v>
+        <v>105.581640076927</v>
       </c>
     </row>
     <row r="16">
@@ -502,7 +502,7 @@
         <v>1992-03</v>
       </c>
       <c r="B16">
-        <v>99.3209260700936</v>
+        <v>99.3208322713877</v>
       </c>
     </row>
     <row r="17">
@@ -510,7 +510,7 @@
         <v>1992-04</v>
       </c>
       <c r="B17">
-        <v>98.5826324806669</v>
+        <v>98.5826550502876</v>
       </c>
     </row>
     <row r="18">
@@ -518,7 +518,7 @@
         <v>1992-05</v>
       </c>
       <c r="B18">
-        <v>100.104081339361</v>
+        <v>100.103864101322</v>
       </c>
     </row>
     <row r="19">
@@ -526,7 +526,7 @@
         <v>1992-06</v>
       </c>
       <c r="B19">
-        <v>101.237513820011</v>
+        <v>101.237489915741</v>
       </c>
     </row>
     <row r="20">
@@ -534,7 +534,7 @@
         <v>1992-07</v>
       </c>
       <c r="B20">
-        <v>93.9868058805159</v>
+        <v>93.9890123221126</v>
       </c>
     </row>
     <row r="21">
@@ -542,7 +542,7 @@
         <v>1992-08</v>
       </c>
       <c r="B21">
-        <v>94.1777467840643</v>
+        <v>94.1839381337934</v>
       </c>
     </row>
     <row r="22">
@@ -550,7 +550,7 @@
         <v>1992-09</v>
       </c>
       <c r="B22">
-        <v>97.2180014077178</v>
+        <v>97.2263806184585</v>
       </c>
     </row>
     <row r="23">
@@ -558,7 +558,7 @@
         <v>1992-10</v>
       </c>
       <c r="B23">
-        <v>92.8448392677847</v>
+        <v>92.8513409791535</v>
       </c>
     </row>
     <row r="24">
@@ -566,7 +566,7 @@
         <v>1992-11</v>
       </c>
       <c r="B24">
-        <v>96.7733866783938</v>
+        <v>96.7872168783841</v>
       </c>
     </row>
     <row r="25">
@@ -574,7 +574,7 @@
         <v>1992-12</v>
       </c>
       <c r="B25">
-        <v>100.071545070885</v>
+        <v>100.087335319536</v>
       </c>
     </row>
     <row r="26">
@@ -582,7 +582,7 @@
         <v>1993-01</v>
       </c>
       <c r="B26">
-        <v>102.310056346894</v>
+        <v>102.318774703091</v>
       </c>
     </row>
     <row r="27">
@@ -590,7 +590,7 @@
         <v>1993-02</v>
       </c>
       <c r="B27">
-        <v>102.054252146104</v>
+        <v>102.072613140367</v>
       </c>
     </row>
     <row r="28">
@@ -598,7 +598,7 @@
         <v>1993-03</v>
       </c>
       <c r="B28">
-        <v>103.025659304853</v>
+        <v>103.045323321714</v>
       </c>
     </row>
     <row r="29">
@@ -606,7 +606,7 @@
         <v>1993-04</v>
       </c>
       <c r="B29">
-        <v>99.2515062862751</v>
+        <v>99.2630036227401</v>
       </c>
     </row>
     <row r="30">
@@ -614,7 +614,7 @@
         <v>1993-05</v>
       </c>
       <c r="B30">
-        <v>101.478781601598</v>
+        <v>101.501508994308</v>
       </c>
     </row>
     <row r="31">
@@ -622,7 +622,7 @@
         <v>1993-06</v>
       </c>
       <c r="B31">
-        <v>104.538889639786</v>
+        <v>104.559815403907</v>
       </c>
     </row>
     <row r="32">
@@ -630,7 +630,7 @@
         <v>1993-07</v>
       </c>
       <c r="B32">
-        <v>105.34879118755</v>
+        <v>105.359303556412</v>
       </c>
     </row>
     <row r="33">
@@ -638,7 +638,7 @@
         <v>1993-08</v>
       </c>
       <c r="B33">
-        <v>105.193018758495</v>
+        <v>105.213429471437</v>
       </c>
     </row>
     <row r="34">
@@ -646,7 +646,7 @@
         <v>1993-09</v>
       </c>
       <c r="B34">
-        <v>110.626354936475</v>
+        <v>110.644318380339</v>
       </c>
     </row>
     <row r="35">
@@ -654,7 +654,7 @@
         <v>1993-10</v>
       </c>
       <c r="B35">
-        <v>111.4683830867</v>
+        <v>111.475538296059</v>
       </c>
     </row>
     <row r="36">
@@ -662,7 +662,7 @@
         <v>1993-11</v>
       </c>
       <c r="B36">
-        <v>114.228391403318</v>
+        <v>114.241950278784</v>
       </c>
     </row>
     <row r="37">
@@ -670,7 +670,7 @@
         <v>1993-12</v>
       </c>
       <c r="B37">
-        <v>114.550880566048</v>
+        <v>114.56261057161</v>
       </c>
     </row>
     <row r="38">
@@ -678,7 +678,7 @@
         <v>1994-01</v>
       </c>
       <c r="B38">
-        <v>108.620724035293</v>
+        <v>108.625528742587</v>
       </c>
     </row>
     <row r="39">
@@ -686,7 +686,7 @@
         <v>1994-02</v>
       </c>
       <c r="B39">
-        <v>121.336604364937</v>
+        <v>121.342728825333</v>
       </c>
     </row>
     <row r="40">
@@ -694,7 +694,7 @@
         <v>1994-03</v>
       </c>
       <c r="B40">
-        <v>118.771890260736</v>
+        <v>118.77738297661</v>
       </c>
     </row>
     <row r="41">
@@ -702,7 +702,7 @@
         <v>1994-04</v>
       </c>
       <c r="B41">
-        <v>114.645111735324</v>
+        <v>114.646278755019</v>
       </c>
     </row>
     <row r="42">
@@ -710,7 +710,7 @@
         <v>1994-05</v>
       </c>
       <c r="B42">
-        <v>116.837748432533</v>
+        <v>116.840390324328</v>
       </c>
     </row>
     <row r="43">
@@ -718,7 +718,7 @@
         <v>1994-06</v>
       </c>
       <c r="B43">
-        <v>110.951098558023</v>
+        <v>110.95303792725</v>
       </c>
     </row>
     <row r="44">
@@ -726,7 +726,7 @@
         <v>1994-07</v>
       </c>
       <c r="B44">
-        <v>107.556262297336</v>
+        <v>107.556039784164</v>
       </c>
     </row>
     <row r="45">
@@ -734,7 +734,7 @@
         <v>1994-08</v>
       </c>
       <c r="B45">
-        <v>110.378907150262</v>
+        <v>110.378001472456</v>
       </c>
     </row>
     <row r="46">
@@ -742,7 +742,7 @@
         <v>1994-09</v>
       </c>
       <c r="B46">
-        <v>105.132871438147</v>
+        <v>105.131582255308</v>
       </c>
     </row>
     <row r="47">
@@ -750,7 +750,7 @@
         <v>1994-10</v>
       </c>
       <c r="B47">
-        <v>104.652911159097</v>
+        <v>104.651381493581</v>
       </c>
     </row>
     <row r="48">
@@ -758,7 +758,7 @@
         <v>1994-11</v>
       </c>
       <c r="B48">
-        <v>106.17787311486</v>
+        <v>106.174843369432</v>
       </c>
     </row>
     <row r="49">
@@ -766,7 +766,7 @@
         <v>1994-12</v>
       </c>
       <c r="B49">
-        <v>105.351306464039</v>
+        <v>105.348035966609</v>
       </c>
     </row>
     <row r="50">
@@ -774,7 +774,7 @@
         <v>1995-01</v>
       </c>
       <c r="B50">
-        <v>94.1868156515358</v>
+        <v>94.1864015824623</v>
       </c>
     </row>
     <row r="51">
@@ -782,7 +782,7 @@
         <v>1995-02</v>
       </c>
       <c r="B51">
-        <v>97.1624369616423</v>
+        <v>97.1606890731794</v>
       </c>
     </row>
     <row r="52">
@@ -790,7 +790,7 @@
         <v>1995-03</v>
       </c>
       <c r="B52">
-        <v>95.6466965994835</v>
+        <v>95.6456907967167</v>
       </c>
     </row>
     <row r="53">
@@ -798,7 +798,7 @@
         <v>1995-04</v>
       </c>
       <c r="B53">
-        <v>91.1540018528607</v>
+        <v>91.154580996063</v>
       </c>
     </row>
     <row r="54">
@@ -806,7 +806,7 @@
         <v>1995-05</v>
       </c>
       <c r="B54">
-        <v>89.726703767894</v>
+        <v>89.7270455099947</v>
       </c>
     </row>
     <row r="55">
@@ -814,7 +814,7 @@
         <v>1995-06</v>
       </c>
       <c r="B55">
-        <v>89.3750132035079</v>
+        <v>89.3749134487088</v>
       </c>
     </row>
     <row r="56">
@@ -822,7 +822,7 @@
         <v>1995-07</v>
       </c>
       <c r="B56">
-        <v>93.3505854842413</v>
+        <v>93.3500808189617</v>
       </c>
     </row>
     <row r="57">
@@ -830,7 +830,7 @@
         <v>1995-08</v>
       </c>
       <c r="B57">
-        <v>94.9465230462235</v>
+        <v>94.9435099042601</v>
       </c>
     </row>
     <row r="58">
@@ -838,7 +838,7 @@
         <v>1995-09</v>
       </c>
       <c r="B58">
-        <v>97.5534099626369</v>
+        <v>97.5485737785067</v>
       </c>
     </row>
     <row r="59">
@@ -846,7 +846,7 @@
         <v>1995-10</v>
       </c>
       <c r="B59">
-        <v>95.0829273896594</v>
+        <v>95.0798681330705</v>
       </c>
     </row>
     <row r="60">
@@ -854,7 +854,7 @@
         <v>1995-11</v>
       </c>
       <c r="B60">
-        <v>96.7497514986346</v>
+        <v>96.7418493374309</v>
       </c>
     </row>
     <row r="61">
@@ -862,7 +862,7 @@
         <v>1995-12</v>
       </c>
       <c r="B61">
-        <v>95.3657272217896</v>
+        <v>95.356770095668</v>
       </c>
     </row>
     <row r="62">
@@ -870,7 +870,7 @@
         <v>1996-01</v>
       </c>
       <c r="B62">
-        <v>100.103109779156</v>
+        <v>100.097233332184</v>
       </c>
     </row>
     <row r="63">
@@ -878,7 +878,7 @@
         <v>1996-02</v>
       </c>
       <c r="B63">
-        <v>95.0085840557888</v>
+        <v>94.9978021297472</v>
       </c>
     </row>
     <row r="64">
@@ -886,7 +886,7 @@
         <v>1996-03</v>
       </c>
       <c r="B64">
-        <v>99.5990183339265</v>
+        <v>99.5868531924489</v>
       </c>
     </row>
     <row r="65">
@@ -894,7 +894,7 @@
         <v>1996-04</v>
       </c>
       <c r="B65">
-        <v>101.117027613172</v>
+        <v>101.109857103938</v>
       </c>
     </row>
     <row r="66">
@@ -902,7 +902,7 @@
         <v>1996-05</v>
       </c>
       <c r="B66">
-        <v>101.595684775058</v>
+        <v>101.582911485509</v>
       </c>
     </row>
     <row r="67">
@@ -910,7 +910,7 @@
         <v>1996-06</v>
       </c>
       <c r="B67">
-        <v>102.338283908569</v>
+        <v>102.325201057249</v>
       </c>
     </row>
     <row r="68">
@@ -918,7 +918,7 @@
         <v>1996-07</v>
       </c>
       <c r="B68">
-        <v>104.494628714592</v>
+        <v>104.486827637643</v>
       </c>
     </row>
     <row r="69">
@@ -926,7 +926,7 @@
         <v>1996-08</v>
       </c>
       <c r="B69">
-        <v>104.122046069039</v>
+        <v>104.107797999031</v>
       </c>
     </row>
     <row r="70">
@@ -934,7 +934,7 @@
         <v>1996-09</v>
       </c>
       <c r="B70">
-        <v>105.870851957291</v>
+        <v>105.856664231958</v>
       </c>
     </row>
     <row r="71">
@@ -942,7 +942,7 @@
         <v>1996-10</v>
       </c>
       <c r="B71">
-        <v>100.945130196232</v>
+        <v>100.93835654638</v>
       </c>
     </row>
     <row r="72">
@@ -950,7 +950,7 @@
         <v>1996-11</v>
       </c>
       <c r="B72">
-        <v>108.818093294906</v>
+        <v>108.804577168948</v>
       </c>
     </row>
     <row r="73">
@@ -958,7 +958,7 @@
         <v>1996-12</v>
       </c>
       <c r="B73">
-        <v>109.198835877813</v>
+        <v>109.185666750339</v>
       </c>
     </row>
     <row r="74">
@@ -966,7 +966,7 @@
         <v>1997-01</v>
       </c>
       <c r="B74">
-        <v>108.71270240078</v>
+        <v>108.70534257261</v>
       </c>
     </row>
     <row r="75">
@@ -974,7 +974,7 @@
         <v>1997-02</v>
       </c>
       <c r="B75">
-        <v>115.62279958051</v>
+        <v>115.609917595108</v>
       </c>
     </row>
     <row r="76">
@@ -982,7 +982,7 @@
         <v>1997-03</v>
       </c>
       <c r="B76">
-        <v>114.393378452963</v>
+        <v>114.381882104483</v>
       </c>
     </row>
     <row r="77">
@@ -990,7 +990,7 @@
         <v>1997-04</v>
       </c>
       <c r="B77">
-        <v>111.105034428606</v>
+        <v>111.098370938667</v>
       </c>
     </row>
     <row r="78">
@@ -998,7 +998,7 @@
         <v>1997-05</v>
       </c>
       <c r="B78">
-        <v>116.949559412476</v>
+        <v>116.938926198121</v>
       </c>
     </row>
     <row r="79">
@@ -1006,7 +1006,7 @@
         <v>1997-06</v>
       </c>
       <c r="B79">
-        <v>113.845926812254</v>
+        <v>113.83597181437</v>
       </c>
     </row>
     <row r="80">
@@ -1014,7 +1014,7 @@
         <v>1997-07</v>
       </c>
       <c r="B80">
-        <v>115.167281573519</v>
+        <v>115.160621745725</v>
       </c>
     </row>
     <row r="81">
@@ -1022,7 +1022,7 @@
         <v>1997-08</v>
       </c>
       <c r="B81">
-        <v>114.683919630745</v>
+        <v>114.673961358001</v>
       </c>
     </row>
     <row r="82">
@@ -1030,7 +1030,7 @@
         <v>1997-09</v>
       </c>
       <c r="B82">
-        <v>117.849854420792</v>
+        <v>117.839029912327</v>
       </c>
     </row>
     <row r="83">
@@ -1038,7 +1038,7 @@
         <v>1997-10</v>
       </c>
       <c r="B83">
-        <v>114.043385693419</v>
+        <v>114.036245519677</v>
       </c>
     </row>
     <row r="84">
@@ -1046,7 +1046,7 @@
         <v>1997-11</v>
       </c>
       <c r="B84">
-        <v>108.798538535515</v>
+        <v>108.787737642015</v>
       </c>
     </row>
     <row r="85">
@@ -1054,7 +1054,7 @@
         <v>1997-12</v>
       </c>
       <c r="B85">
-        <v>108.855216389211</v>
+        <v>108.843506045726</v>
       </c>
     </row>
     <row r="86">
@@ -1062,7 +1062,7 @@
         <v>1998-01</v>
       </c>
       <c r="B86">
-        <v>106.105434314756</v>
+        <v>106.098074545395</v>
       </c>
     </row>
     <row r="87">
@@ -1070,7 +1070,7 @@
         <v>1998-02</v>
       </c>
       <c r="B87">
-        <v>102.970540710769</v>
+        <v>102.958324322554</v>
       </c>
     </row>
     <row r="88">
@@ -1078,7 +1078,7 @@
         <v>1998-03</v>
       </c>
       <c r="B88">
-        <v>106.138214608689</v>
+        <v>106.125014557837</v>
       </c>
     </row>
     <row r="89">
@@ -1086,7 +1086,7 @@
         <v>1998-04</v>
       </c>
       <c r="B89">
-        <v>104.803438137237</v>
+        <v>104.795552731994</v>
       </c>
     </row>
     <row r="90">
@@ -1094,7 +1094,7 @@
         <v>1998-05</v>
       </c>
       <c r="B90">
-        <v>109.27833839903</v>
+        <v>109.263660530326</v>
       </c>
     </row>
     <row r="91">
@@ -1102,7 +1102,7 @@
         <v>1998-06</v>
       </c>
       <c r="B91">
-        <v>102.142645066214</v>
+        <v>102.12952643196</v>
       </c>
     </row>
     <row r="92">
@@ -1110,7 +1110,7 @@
         <v>1998-07</v>
       </c>
       <c r="B92">
-        <v>105.090744883348</v>
+        <v>105.082961755968</v>
       </c>
     </row>
     <row r="93">
@@ -1118,7 +1118,7 @@
         <v>1998-08</v>
       </c>
       <c r="B93">
-        <v>101.012079313024</v>
+        <v>101.00031874308</v>
       </c>
     </row>
     <row r="94">
@@ -1126,7 +1126,7 @@
         <v>1998-09</v>
       </c>
       <c r="B94">
-        <v>99.5065198977626</v>
+        <v>99.4953689392215</v>
       </c>
     </row>
     <row r="95">
@@ -1134,7 +1134,7 @@
         <v>1998-10</v>
       </c>
       <c r="B95">
-        <v>98.8675194759678</v>
+        <v>98.8614928472161</v>
       </c>
     </row>
     <row r="96">
@@ -1142,7 +1142,7 @@
         <v>1998-11</v>
       </c>
       <c r="B96">
-        <v>96.2731840980958</v>
+        <v>96.2633825305662</v>
       </c>
     </row>
     <row r="97">
@@ -1150,7 +1150,7 @@
         <v>1998-12</v>
       </c>
       <c r="B97">
-        <v>96.6104073973002</v>
+        <v>96.6010353468968</v>
       </c>
     </row>
     <row r="98">
@@ -1158,7 +1158,7 @@
         <v>1999-01</v>
       </c>
       <c r="B98">
-        <v>100.344962493553</v>
+        <v>100.339525847491</v>
       </c>
     </row>
     <row r="99">
@@ -1166,7 +1166,7 @@
         <v>1999-02</v>
       </c>
       <c r="B99">
-        <v>98.2654711376889</v>
+        <v>98.2571761321402</v>
       </c>
     </row>
     <row r="100">
@@ -1174,7 +1174,7 @@
         <v>1999-03</v>
       </c>
       <c r="B100">
-        <v>98.6612634292648</v>
+        <v>98.6541396013365</v>
       </c>
     </row>
     <row r="101">
@@ -1182,7 +1182,7 @@
         <v>1999-04</v>
       </c>
       <c r="B101">
-        <v>103.353470879833</v>
+        <v>103.349464756304</v>
       </c>
     </row>
     <row r="102">
@@ -1190,7 +1190,7 @@
         <v>1999-05</v>
       </c>
       <c r="B102">
-        <v>103.958539904442</v>
+        <v>103.954228358599</v>
       </c>
     </row>
     <row r="103">
@@ -1198,7 +1198,7 @@
         <v>1999-06</v>
       </c>
       <c r="B103">
-        <v>106.054032632918</v>
+        <v>106.050493809217</v>
       </c>
     </row>
     <row r="104">
@@ -1206,7 +1206,7 @@
         <v>1999-07</v>
       </c>
       <c r="B104">
-        <v>105.408448243345</v>
+        <v>105.406749372293</v>
       </c>
     </row>
     <row r="105">
@@ -1214,7 +1214,7 @@
         <v>1999-08</v>
       </c>
       <c r="B105">
-        <v>108.388724622781</v>
+        <v>108.38709193762</v>
       </c>
     </row>
     <row r="106">
@@ -1222,7 +1222,7 @@
         <v>1999-09</v>
       </c>
       <c r="B106">
-        <v>107.174104410249</v>
+        <v>107.173452568817</v>
       </c>
     </row>
     <row r="107">
@@ -1230,7 +1230,7 @@
         <v>1999-10</v>
       </c>
       <c r="B107">
-        <v>108.285179197924</v>
+        <v>108.284395229468</v>
       </c>
     </row>
     <row r="108">
@@ -1238,7 +1238,7 @@
         <v>1999-11</v>
       </c>
       <c r="B108">
-        <v>112.429716438279</v>
+        <v>112.429066315336</v>
       </c>
     </row>
     <row r="109">
@@ -1246,7 +1246,7 @@
         <v>1999-12</v>
       </c>
       <c r="B109">
-        <v>110.852603549985</v>
+        <v>110.852313027214</v>
       </c>
     </row>
     <row r="110">
@@ -1254,7 +1254,7 @@
         <v>2000-01</v>
       </c>
       <c r="B110">
-        <v>107.890206237484</v>
+        <v>107.889734907708</v>
       </c>
     </row>
     <row r="111">
@@ -1262,7 +1262,7 @@
         <v>2000-02</v>
       </c>
       <c r="B111">
-        <v>106.90950737368</v>
+        <v>106.909523694315</v>
       </c>
     </row>
     <row r="112">
@@ -1270,7 +1270,7 @@
         <v>2000-03</v>
       </c>
       <c r="B112">
-        <v>109.735255270536</v>
+        <v>109.735037746962</v>
       </c>
     </row>
     <row r="113">
@@ -1278,7 +1278,7 @@
         <v>2000-04</v>
       </c>
       <c r="B113">
-        <v>108.639333496626</v>
+        <v>108.638805665106</v>
       </c>
     </row>
     <row r="114">
@@ -1286,7 +1286,7 @@
         <v>2000-05</v>
       </c>
       <c r="B114">
-        <v>106.129187019898</v>
+        <v>106.129962821058</v>
       </c>
     </row>
     <row r="115">
@@ -1294,7 +1294,7 @@
         <v>2000-06</v>
       </c>
       <c r="B115">
-        <v>107.121768155241</v>
+        <v>107.122619247855</v>
       </c>
     </row>
     <row r="116">
@@ -1302,7 +1302,7 @@
         <v>2000-07</v>
       </c>
       <c r="B116">
-        <v>103.691808468641</v>
+        <v>103.692419989754</v>
       </c>
     </row>
     <row r="117">
@@ -1310,7 +1310,7 @@
         <v>2000-08</v>
       </c>
       <c r="B117">
-        <v>98.6717757199777</v>
+        <v>98.6737763140078</v>
       </c>
     </row>
     <row r="118">
@@ -1318,7 +1318,7 @@
         <v>2000-09</v>
       </c>
       <c r="B118">
-        <v>98.1029077663998</v>
+        <v>98.10443010812</v>
       </c>
     </row>
     <row r="119">
@@ -1326,7 +1326,7 @@
         <v>2000-10</v>
       </c>
       <c r="B119">
-        <v>100.316850026187</v>
+        <v>100.316842751392</v>
       </c>
     </row>
     <row r="120">
@@ -1334,7 +1334,7 @@
         <v>2000-11</v>
       </c>
       <c r="B120">
-        <v>99.2314230111561</v>
+        <v>99.2302652207187</v>
       </c>
     </row>
     <row r="121">
@@ -1342,7 +1342,7 @@
         <v>2000-12</v>
       </c>
       <c r="B121">
-        <v>96.4926320473327</v>
+        <v>96.489931740163</v>
       </c>
     </row>
     <row r="122">
@@ -1350,7 +1350,7 @@
         <v>2001-01</v>
       </c>
       <c r="B122">
-        <v>94.3961919647907</v>
+        <v>94.3933661254196</v>
       </c>
     </row>
     <row r="123">
@@ -1358,7 +1358,7 @@
         <v>2001-02</v>
       </c>
       <c r="B123">
-        <v>86.1297082867929</v>
+        <v>86.1235303075857</v>
       </c>
     </row>
     <row r="124">
@@ -1366,7 +1366,7 @@
         <v>2001-03</v>
       </c>
       <c r="B124">
-        <v>84.8850532989555</v>
+        <v>84.87616548429</v>
       </c>
     </row>
     <row r="125">
@@ -1374,7 +1374,7 @@
         <v>2001-04</v>
       </c>
       <c r="B125">
-        <v>90.4043064379889</v>
+        <v>90.3971725211827</v>
       </c>
     </row>
     <row r="126">
@@ -1382,7 +1382,7 @@
         <v>2001-05</v>
       </c>
       <c r="B126">
-        <v>85.9489453670756</v>
+        <v>85.9320054163338</v>
       </c>
     </row>
     <row r="127">
@@ -1390,7 +1390,7 @@
         <v>2001-06</v>
       </c>
       <c r="B127">
-        <v>91.0560339074409</v>
+        <v>91.0369956808038</v>
       </c>
     </row>
     <row r="128">
@@ -1398,7 +1398,7 @@
         <v>2001-07</v>
       </c>
       <c r="B128">
-        <v>89.1969988095455</v>
+        <v>89.1867479178355</v>
       </c>
     </row>
     <row r="129">
@@ -1406,7 +1406,7 @@
         <v>2001-08</v>
       </c>
       <c r="B129">
-        <v>90.5654951537513</v>
+        <v>90.5487915002313</v>
       </c>
     </row>
     <row r="130">
@@ -1414,7 +1414,7 @@
         <v>2001-09</v>
       </c>
       <c r="B130">
-        <v>87.7999304944093</v>
+        <v>87.7871168619801</v>
       </c>
     </row>
     <row r="131">
@@ -1422,7 +1422,7 @@
         <v>2001-10</v>
       </c>
       <c r="B131">
-        <v>80.8280681597171</v>
+        <v>80.8239069295415</v>
       </c>
     </row>
     <row r="132">
@@ -1430,7 +1430,7 @@
         <v>2001-11</v>
       </c>
       <c r="B132">
-        <v>83.2242071283395</v>
+        <v>83.2171465347706</v>
       </c>
     </row>
     <row r="133">
@@ -1438,7 +1438,7 @@
         <v>2001-12</v>
       </c>
       <c r="B133">
-        <v>85.4500688815673</v>
+        <v>85.4456882712221</v>
       </c>
     </row>
     <row r="134">
@@ -1446,7 +1446,7 @@
         <v>2002-01</v>
       </c>
       <c r="B134">
-        <v>91.6252950646791</v>
+        <v>91.6237277045958</v>
       </c>
     </row>
     <row r="135">
@@ -1454,7 +1454,7 @@
         <v>2002-02</v>
       </c>
       <c r="B135">
-        <v>96.5385505279724</v>
+        <v>96.5356039078296</v>
       </c>
     </row>
     <row r="136">
@@ -1462,7 +1462,7 @@
         <v>2002-03</v>
       </c>
       <c r="B136">
-        <v>99.0147068512242</v>
+        <v>99.0128469298936</v>
       </c>
     </row>
     <row r="137">
@@ -1470,7 +1470,7 @@
         <v>2002-04</v>
       </c>
       <c r="B137">
-        <v>100.622246935188</v>
+        <v>100.62161343846</v>
       </c>
     </row>
     <row r="138">
@@ -1478,7 +1478,7 @@
         <v>2002-05</v>
       </c>
       <c r="B138">
-        <v>100.056755940317</v>
+        <v>100.057262001773</v>
       </c>
     </row>
     <row r="139">
@@ -1486,7 +1486,7 @@
         <v>2002-06</v>
       </c>
       <c r="B139">
-        <v>98.9648853032681</v>
+        <v>98.96574323363</v>
       </c>
     </row>
     <row r="140">
@@ -1494,7 +1494,7 @@
         <v>2002-07</v>
       </c>
       <c r="B140">
-        <v>95.8434516194321</v>
+        <v>95.8449872205129</v>
       </c>
     </row>
     <row r="141">
@@ -1502,7 +1502,7 @@
         <v>2002-08</v>
       </c>
       <c r="B141">
-        <v>94.6911207955795</v>
+        <v>94.6930539757931</v>
       </c>
     </row>
     <row r="142">
@@ -1510,7 +1510,7 @@
         <v>2002-09</v>
       </c>
       <c r="B142">
-        <v>96.7825376733545</v>
+        <v>96.7845391676858</v>
       </c>
     </row>
     <row r="143">
@@ -1518,7 +1518,7 @@
         <v>2002-10</v>
       </c>
       <c r="B143">
-        <v>97.6265778223052</v>
+        <v>97.6277282253926</v>
       </c>
     </row>
     <row r="144">
@@ -1526,7 +1526,7 @@
         <v>2002-11</v>
       </c>
       <c r="B144">
-        <v>100.477089833826</v>
+        <v>100.477943039287</v>
       </c>
     </row>
     <row r="145">
@@ -1534,7 +1534,7 @@
         <v>2002-12</v>
       </c>
       <c r="B145">
-        <v>101.940946594569</v>
+        <v>101.941585120583</v>
       </c>
     </row>
     <row r="146">
@@ -1542,7 +1542,7 @@
         <v>2003-01</v>
       </c>
       <c r="B146">
-        <v>96.4902732491999</v>
+        <v>96.4913834070017</v>
       </c>
     </row>
     <row r="147">
@@ -1550,7 +1550,7 @@
         <v>2003-02</v>
       </c>
       <c r="B147">
-        <v>92.7989094789193</v>
+        <v>92.8018243245578</v>
       </c>
     </row>
     <row r="148">
@@ -1558,7 +1558,7 @@
         <v>2003-03</v>
       </c>
       <c r="B148">
-        <v>90.5021502968263</v>
+        <v>90.5054831743798</v>
       </c>
     </row>
     <row r="149">
@@ -1566,7 +1566,7 @@
         <v>2003-04</v>
       </c>
       <c r="B149">
-        <v>90.7598254065192</v>
+        <v>90.762150945377</v>
       </c>
     </row>
     <row r="150">
@@ -1574,7 +1574,7 @@
         <v>2003-05</v>
       </c>
       <c r="B150">
-        <v>93.0283784848179</v>
+        <v>93.0309627120577</v>
       </c>
     </row>
     <row r="151">
@@ -1582,7 +1582,7 @@
         <v>2003-06</v>
       </c>
       <c r="B151">
-        <v>93.5497210022401</v>
+        <v>93.5527579077748</v>
       </c>
     </row>
     <row r="152">
@@ -1590,7 +1590,7 @@
         <v>2003-07</v>
       </c>
       <c r="B152">
-        <v>101.290964005547</v>
+        <v>101.291688491685</v>
       </c>
     </row>
     <row r="153">
@@ -1598,7 +1598,7 @@
         <v>2003-08</v>
       </c>
       <c r="B153">
-        <v>104.082287902118</v>
+        <v>104.084046978991</v>
       </c>
     </row>
     <row r="154">
@@ -1606,7 +1606,7 @@
         <v>2003-09</v>
       </c>
       <c r="B154">
-        <v>107.605666208142</v>
+        <v>107.606166423104</v>
       </c>
     </row>
     <row r="155">
@@ -1614,7 +1614,7 @@
         <v>2003-10</v>
       </c>
       <c r="B155">
-        <v>109.062865296517</v>
+        <v>109.062486480871</v>
       </c>
     </row>
     <row r="156">
@@ -1622,7 +1622,7 @@
         <v>2003-11</v>
       </c>
       <c r="B156">
-        <v>109.320223243075</v>
+        <v>109.31997465956</v>
       </c>
     </row>
     <row r="157">
@@ -1630,7 +1630,7 @@
         <v>2003-12</v>
       </c>
       <c r="B157">
-        <v>109.148309897435</v>
+        <v>109.149289995001</v>
       </c>
     </row>
     <row r="158">
@@ -1638,7 +1638,7 @@
         <v>2004-01</v>
       </c>
       <c r="B158">
-        <v>110.271253828278</v>
+        <v>110.270632433839</v>
       </c>
     </row>
     <row r="159">
@@ -1646,7 +1646,7 @@
         <v>2004-02</v>
       </c>
       <c r="B159">
-        <v>109.364057641512</v>
+        <v>109.364298279715</v>
       </c>
     </row>
     <row r="160">
@@ -1654,7 +1654,7 @@
         <v>2004-03</v>
       </c>
       <c r="B160">
-        <v>111.603605695216</v>
+        <v>111.603168889103</v>
       </c>
     </row>
     <row r="161">
@@ -1662,7 +1662,7 @@
         <v>2004-04</v>
       </c>
       <c r="B161">
-        <v>113.32520667206</v>
+        <v>113.322928298072</v>
       </c>
     </row>
     <row r="162">
@@ -1670,7 +1670,7 @@
         <v>2004-05</v>
       </c>
       <c r="B162">
-        <v>111.219066088104</v>
+        <v>111.218488864278</v>
       </c>
     </row>
     <row r="163">
@@ -1678,7 +1678,7 @@
         <v>2004-06</v>
       </c>
       <c r="B163">
-        <v>108.580505607953</v>
+        <v>108.579456160568</v>
       </c>
     </row>
     <row r="164">
@@ -1686,7 +1686,7 @@
         <v>2004-07</v>
       </c>
       <c r="B164">
-        <v>106.833107490714</v>
+        <v>106.831857330051</v>
       </c>
     </row>
     <row r="165">
@@ -1694,7 +1694,7 @@
         <v>2004-08</v>
       </c>
       <c r="B165">
-        <v>105.317333112696</v>
+        <v>105.315739387839</v>
       </c>
     </row>
     <row r="166">
@@ -1702,7 +1702,7 @@
         <v>2004-09</v>
       </c>
       <c r="B166">
-        <v>102.591968038286</v>
+        <v>102.590494879003</v>
       </c>
     </row>
     <row r="167">
@@ -1710,7 +1710,7 @@
         <v>2004-10</v>
       </c>
       <c r="B167">
-        <v>102.928983341001</v>
+        <v>102.927885454624</v>
       </c>
     </row>
     <row r="168">
@@ -1718,7 +1718,7 @@
         <v>2004-11</v>
       </c>
       <c r="B168">
-        <v>98.497306133358</v>
+        <v>98.4960076894898</v>
       </c>
     </row>
     <row r="169">
@@ -1726,7 +1726,7 @@
         <v>2004-12</v>
       </c>
       <c r="B169">
-        <v>97.2603481141648</v>
+        <v>97.2594910998608</v>
       </c>
     </row>
     <row r="170">
@@ -1734,7 +1734,7 @@
         <v>2005-01</v>
       </c>
       <c r="B170">
-        <v>97.1469192959439</v>
+        <v>97.1466836449853</v>
       </c>
     </row>
     <row r="171">
@@ -1742,7 +1742,7 @@
         <v>2005-02</v>
       </c>
       <c r="B171">
-        <v>100.25775268928</v>
+        <v>100.256979755902</v>
       </c>
     </row>
     <row r="172">
@@ -1750,7 +1750,7 @@
         <v>2005-03</v>
       </c>
       <c r="B172">
-        <v>98.5903647320539</v>
+        <v>98.5896834237513</v>
       </c>
     </row>
     <row r="173">
@@ -1758,7 +1758,7 @@
         <v>2005-04</v>
       </c>
       <c r="B173">
-        <v>99.7180326081011</v>
+        <v>99.718150236634</v>
       </c>
     </row>
     <row r="174">
@@ -1766,7 +1766,7 @@
         <v>2005-05</v>
       </c>
       <c r="B174">
-        <v>99.5982718890436</v>
+        <v>99.5968617031422</v>
       </c>
     </row>
     <row r="175">
@@ -1774,7 +1774,7 @@
         <v>2005-06</v>
       </c>
       <c r="B175">
-        <v>100.220110746072</v>
+        <v>100.218630484471</v>
       </c>
     </row>
     <row r="176">
@@ -1782,7 +1782,7 @@
         <v>2005-07</v>
       </c>
       <c r="B176">
-        <v>102.634976121132</v>
+        <v>102.633726902884</v>
       </c>
     </row>
     <row r="177">
@@ -1790,7 +1790,7 @@
         <v>2005-08</v>
       </c>
       <c r="B177">
-        <v>103.197464718976</v>
+        <v>103.195438577985</v>
       </c>
     </row>
     <row r="178">
@@ -1798,7 +1798,7 @@
         <v>2005-09</v>
       </c>
       <c r="B178">
-        <v>105.989852541993</v>
+        <v>105.987768493921</v>
       </c>
     </row>
     <row r="179">
@@ -1806,7 +1806,7 @@
         <v>2005-10</v>
       </c>
       <c r="B179">
-        <v>108.1613720905</v>
+        <v>108.159119763699</v>
       </c>
     </row>
     <row r="180">
@@ -1814,7 +1814,7 @@
         <v>2005-11</v>
       </c>
       <c r="B180">
-        <v>107.484096972966</v>
+        <v>107.481592223679</v>
       </c>
     </row>
     <row r="181">
@@ -1822,7 +1822,7 @@
         <v>2005-12</v>
       </c>
       <c r="B181">
-        <v>106.203461377914</v>
+        <v>106.200685773564</v>
       </c>
     </row>
     <row r="182">
@@ -1830,7 +1830,7 @@
         <v>2006-01</v>
       </c>
       <c r="B182">
-        <v>108.70752814456</v>
+        <v>108.705031332075</v>
       </c>
     </row>
     <row r="183">
@@ -1838,7 +1838,7 @@
         <v>2006-02</v>
       </c>
       <c r="B183">
-        <v>108.798664374048</v>
+        <v>108.794904916209</v>
       </c>
     </row>
     <row r="184">
@@ -1846,7 +1846,7 @@
         <v>2006-03</v>
       </c>
       <c r="B184">
-        <v>107.586463015185</v>
+        <v>107.583676431014</v>
       </c>
     </row>
     <row r="185">
@@ -1854,7 +1854,7 @@
         <v>2006-04</v>
       </c>
       <c r="B185">
-        <v>109.683918936908</v>
+        <v>109.681454177611</v>
       </c>
     </row>
     <row r="186">
@@ -1862,7 +1862,7 @@
         <v>2006-05</v>
       </c>
       <c r="B186">
-        <v>107.864445596258</v>
+        <v>107.862389682634</v>
       </c>
     </row>
     <row r="187">
@@ -1870,7 +1870,7 @@
         <v>2006-06</v>
       </c>
       <c r="B187">
-        <v>107.493767474747</v>
+        <v>107.491563695479</v>
       </c>
     </row>
     <row r="188">
@@ -1878,7 +1878,7 @@
         <v>2006-07</v>
       </c>
       <c r="B188">
-        <v>104.350612467224</v>
+        <v>104.3495184928</v>
       </c>
     </row>
     <row r="189">
@@ -1886,7 +1886,7 @@
         <v>2006-08</v>
       </c>
       <c r="B189">
-        <v>104.796953295684</v>
+        <v>104.796301408567</v>
       </c>
     </row>
     <row r="190">
@@ -1894,7 +1894,7 @@
         <v>2006-09</v>
       </c>
       <c r="B190">
-        <v>102.808920998638</v>
+        <v>102.808536951515</v>
       </c>
     </row>
     <row r="191">
@@ -1902,7 +1902,7 @@
         <v>2006-10</v>
       </c>
       <c r="B191">
-        <v>104.242214594761</v>
+        <v>104.241923677238</v>
       </c>
     </row>
     <row r="192">
@@ -1910,7 +1910,7 @@
         <v>2006-11</v>
       </c>
       <c r="B192">
-        <v>106.395951524292</v>
+        <v>106.396251305883</v>
       </c>
     </row>
     <row r="193">
@@ -1918,7 +1918,7 @@
         <v>2006-12</v>
       </c>
       <c r="B193">
-        <v>108.226429613899</v>
+        <v>108.227859640063</v>
       </c>
     </row>
     <row r="194">
@@ -1926,7 +1926,7 @@
         <v>2007-01</v>
       </c>
       <c r="B194">
-        <v>106.097627854116</v>
+        <v>106.098487373377</v>
       </c>
     </row>
     <row r="195">
@@ -1934,7 +1934,7 @@
         <v>2007-02</v>
       </c>
       <c r="B195">
-        <v>103.789511076149</v>
+        <v>103.793126776886</v>
       </c>
     </row>
     <row r="196">
@@ -1942,7 +1942,7 @@
         <v>2007-03</v>
       </c>
       <c r="B196">
-        <v>103.939589361144</v>
+        <v>103.94386126347</v>
       </c>
     </row>
     <row r="197">
@@ -1950,7 +1950,7 @@
         <v>2007-04</v>
       </c>
       <c r="B197">
-        <v>100.907881351464</v>
+        <v>100.911553335723</v>
       </c>
     </row>
     <row r="198">
@@ -1958,7 +1958,7 @@
         <v>2007-05</v>
       </c>
       <c r="B198">
-        <v>99.300564404543</v>
+        <v>99.3068085961925</v>
       </c>
     </row>
     <row r="199">
@@ -1966,7 +1966,7 @@
         <v>2007-06</v>
       </c>
       <c r="B199">
-        <v>101.484526505727</v>
+        <v>101.492141291422</v>
       </c>
     </row>
     <row r="200">
@@ -1974,7 +1974,7 @@
         <v>2007-07</v>
       </c>
       <c r="B200">
-        <v>101.457113153365</v>
+        <v>101.462234224647</v>
       </c>
     </row>
     <row r="201">
@@ -1982,7 +1982,7 @@
         <v>2007-08</v>
       </c>
       <c r="B201">
-        <v>99.7381580867158</v>
+        <v>99.7472190731887</v>
       </c>
     </row>
     <row r="202">
@@ -1990,7 +1990,7 @@
         <v>2007-09</v>
       </c>
       <c r="B202">
-        <v>102.807381340485</v>
+        <v>102.817003842523</v>
       </c>
     </row>
     <row r="203">
@@ -1998,7 +1998,7 @@
         <v>2007-10</v>
       </c>
       <c r="B203">
-        <v>98.5154540662902</v>
+        <v>98.5220181164174</v>
       </c>
     </row>
     <row r="204">
@@ -2006,7 +2006,7 @@
         <v>2007-11</v>
       </c>
       <c r="B204">
-        <v>98.7769783947203</v>
+        <v>98.7869402680862</v>
       </c>
     </row>
     <row r="205">
@@ -2014,7 +2014,7 @@
         <v>2007-12</v>
       </c>
       <c r="B205">
-        <v>97.5790702517176</v>
+        <v>97.5890739202705</v>
       </c>
     </row>
     <row r="206">
@@ -2022,7 +2022,7 @@
         <v>2008-01</v>
       </c>
       <c r="B206">
-        <v>98.9248129622749</v>
+        <v>98.9303895405667</v>
       </c>
     </row>
     <row r="207">
@@ -2030,7 +2030,7 @@
         <v>2008-02</v>
       </c>
       <c r="B207">
-        <v>95.431062049445</v>
+        <v>95.4386937563348</v>
       </c>
     </row>
     <row r="208">
@@ -2038,7 +2038,7 @@
         <v>2008-03</v>
       </c>
       <c r="B208">
-        <v>92.3530264208359</v>
+        <v>92.359555157981</v>
       </c>
     </row>
     <row r="209">
@@ -2046,7 +2046,7 @@
         <v>2008-04</v>
       </c>
       <c r="B209">
-        <v>91.2888646816241</v>
+        <v>91.2917953207025</v>
       </c>
     </row>
     <row r="210">
@@ -2054,7 +2054,7 @@
         <v>2008-05</v>
       </c>
       <c r="B210">
-        <v>93.4287350758417</v>
+        <v>93.4313916880285</v>
       </c>
     </row>
     <row r="211">
@@ -2062,7 +2062,7 @@
         <v>2008-06</v>
       </c>
       <c r="B211">
-        <v>91.2294350619265</v>
+        <v>91.2304362401756</v>
       </c>
     </row>
     <row r="212">
@@ -2070,7 +2070,7 @@
         <v>2008-07</v>
       </c>
       <c r="B212">
-        <v>90.9854748001244</v>
+        <v>90.9852281570592</v>
       </c>
     </row>
     <row r="213">
@@ -2078,7 +2078,7 @@
         <v>2008-08</v>
       </c>
       <c r="B213">
-        <v>88.1691827892724</v>
+        <v>88.166664716602</v>
       </c>
     </row>
     <row r="214">
@@ -2086,7 +2086,7 @@
         <v>2008-09</v>
       </c>
       <c r="B214">
-        <v>84.6851250442795</v>
+        <v>84.6809620226799</v>
       </c>
     </row>
     <row r="215">
@@ -2094,7 +2094,7 @@
         <v>2008-10</v>
       </c>
       <c r="B215">
-        <v>83.899164361492</v>
+        <v>83.896449726251</v>
       </c>
     </row>
     <row r="216">
@@ -2102,7 +2102,7 @@
         <v>2008-11</v>
       </c>
       <c r="B216">
-        <v>77.9528222283534</v>
+        <v>77.9473251427495</v>
       </c>
     </row>
     <row r="217">
@@ -2110,7 +2110,7 @@
         <v>2008-12</v>
       </c>
       <c r="B217">
-        <v>75.3864125105167</v>
+        <v>75.3804041558227</v>
       </c>
     </row>
     <row r="218">
@@ -2118,7 +2118,7 @@
         <v>2009-01</v>
       </c>
       <c r="B218">
-        <v>74.4034095824518</v>
+        <v>74.4004486450921</v>
       </c>
     </row>
     <row r="219">
@@ -2126,7 +2126,7 @@
         <v>2009-02</v>
       </c>
       <c r="B219">
-        <v>76.1265695777928</v>
+        <v>76.1201135297349</v>
       </c>
     </row>
     <row r="220">
@@ -2134,7 +2134,7 @@
         <v>2009-03</v>
       </c>
       <c r="B220">
-        <v>79.0430976617172</v>
+        <v>79.0363464382953</v>
       </c>
     </row>
     <row r="221">
@@ -2142,7 +2142,7 @@
         <v>2009-04</v>
       </c>
       <c r="B221">
-        <v>82.3494781538038</v>
+        <v>82.3469351996802</v>
       </c>
     </row>
     <row r="222">
@@ -2150,7 +2150,7 @@
         <v>2009-05</v>
       </c>
       <c r="B222">
-        <v>92.6407589740579</v>
+        <v>92.6345185849647</v>
       </c>
     </row>
     <row r="223">
@@ -2158,7 +2158,7 @@
         <v>2009-06</v>
       </c>
       <c r="B223">
-        <v>96.1290050956664</v>
+        <v>96.123380816401</v>
       </c>
     </row>
     <row r="224">
@@ -2166,7 +2166,7 @@
         <v>2009-07</v>
       </c>
       <c r="B224">
-        <v>98.049260250253</v>
+        <v>98.0464073564827</v>
       </c>
     </row>
     <row r="225">
@@ -2174,7 +2174,7 @@
         <v>2009-08</v>
       </c>
       <c r="B225">
-        <v>103.055692476669</v>
+        <v>103.051925711113</v>
       </c>
     </row>
     <row r="226">
@@ -2182,7 +2182,7 @@
         <v>2009-09</v>
       </c>
       <c r="B226">
-        <v>108.14896765873</v>
+        <v>108.146253803255</v>
       </c>
     </row>
     <row r="227">
@@ -2190,7 +2190,7 @@
         <v>2009-10</v>
       </c>
       <c r="B227">
-        <v>108.906075854353</v>
+        <v>108.904529176294</v>
       </c>
     </row>
     <row r="228">
@@ -2198,7 +2198,7 @@
         <v>2009-11</v>
       </c>
       <c r="B228">
-        <v>111.42454011452</v>
+        <v>111.423478256886</v>
       </c>
     </row>
     <row r="229">
@@ -2206,7 +2206,7 @@
         <v>2009-12</v>
       </c>
       <c r="B229">
-        <v>113.202697260643</v>
+        <v>113.201798091675</v>
       </c>
     </row>
     <row r="230">
@@ -2214,7 +2214,7 @@
         <v>2010-01</v>
       </c>
       <c r="B230">
-        <v>108.786245671611</v>
+        <v>108.78637119848</v>
       </c>
     </row>
     <row r="231">
@@ -2222,7 +2222,7 @@
         <v>2010-02</v>
       </c>
       <c r="B231">
-        <v>116.908397476258</v>
+        <v>116.908050651639</v>
       </c>
     </row>
     <row r="232">
@@ -2230,7 +2230,7 @@
         <v>2010-03</v>
       </c>
       <c r="B232">
-        <v>115.193824086328</v>
+        <v>115.194099230532</v>
       </c>
     </row>
     <row r="233">
@@ -2238,7 +2238,7 @@
         <v>2010-04</v>
       </c>
       <c r="B233">
-        <v>114.374129347643</v>
+        <v>114.37340324595</v>
       </c>
     </row>
     <row r="234">
@@ -2246,7 +2246,7 @@
         <v>2010-05</v>
       </c>
       <c r="B234">
-        <v>113.410918177735</v>
+        <v>113.411264541366</v>
       </c>
     </row>
     <row r="235">
@@ -2254,7 +2254,7 @@
         <v>2010-06</v>
       </c>
       <c r="B235">
-        <v>112.618072021951</v>
+        <v>112.618091649622</v>
       </c>
     </row>
     <row r="236">
@@ -2262,7 +2262,7 @@
         <v>2010-07</v>
       </c>
       <c r="B236">
-        <v>111.730703031092</v>
+        <v>111.729850870603</v>
       </c>
     </row>
     <row r="237">
@@ -2270,7 +2270,7 @@
         <v>2010-08</v>
       </c>
       <c r="B237">
-        <v>107.676465750479</v>
+        <v>107.676737099363</v>
       </c>
     </row>
     <row r="238">
@@ -2278,7 +2278,7 @@
         <v>2010-09</v>
       </c>
       <c r="B238">
-        <v>104.302013436442</v>
+        <v>104.302324786628</v>
       </c>
     </row>
     <row r="239">
@@ -2286,7 +2286,7 @@
         <v>2010-10</v>
       </c>
       <c r="B239">
-        <v>103.980544220377</v>
+        <v>103.980730605721</v>
       </c>
     </row>
     <row r="240">
@@ -2294,7 +2294,7 @@
         <v>2010-11</v>
       </c>
       <c r="B240">
-        <v>103.491815942082</v>
+        <v>103.49319117779</v>
       </c>
     </row>
     <row r="241">
@@ -2302,7 +2302,7 @@
         <v>2010-12</v>
       </c>
       <c r="B241">
-        <v>101.142197966727</v>
+        <v>101.144304978893</v>
       </c>
     </row>
     <row r="242">
@@ -2310,7 +2310,7 @@
         <v>2011-01</v>
       </c>
       <c r="B242">
-        <v>100.841614694887</v>
+        <v>100.842786523461</v>
       </c>
     </row>
     <row r="243">
@@ -2318,7 +2318,7 @@
         <v>2011-02</v>
       </c>
       <c r="B243">
-        <v>98.0089312645558</v>
+        <v>98.0121543803849</v>
       </c>
     </row>
     <row r="244">
@@ -2326,7 +2326,7 @@
         <v>2011-03</v>
       </c>
       <c r="B244">
-        <v>100.044847146686</v>
+        <v>100.047423545624</v>
       </c>
     </row>
     <row r="245">
@@ -2334,7 +2334,7 @@
         <v>2011-04</v>
       </c>
       <c r="B245">
-        <v>100.058862168836</v>
+        <v>100.060382906253</v>
       </c>
     </row>
     <row r="246">
@@ -2342,7 +2342,7 @@
         <v>2011-05</v>
       </c>
       <c r="B246">
-        <v>96.2152575991172</v>
+        <v>96.2178050248717</v>
       </c>
     </row>
     <row r="247">
@@ -2350,7 +2350,7 @@
         <v>2011-06</v>
       </c>
       <c r="B247">
-        <v>93.8435119684165</v>
+        <v>93.8464348446071</v>
       </c>
     </row>
     <row r="248">
@@ -2358,7 +2358,7 @@
         <v>2011-07</v>
       </c>
       <c r="B248">
-        <v>88.5376902288564</v>
+        <v>88.5402703567009</v>
       </c>
     </row>
     <row r="249">
@@ -2366,7 +2366,7 @@
         <v>2011-08</v>
       </c>
       <c r="B249">
-        <v>84.864537094297</v>
+        <v>84.868039944036</v>
       </c>
     </row>
     <row r="250">
@@ -2374,7 +2374,7 @@
         <v>2011-09</v>
       </c>
       <c r="B250">
-        <v>84.640522525665</v>
+        <v>84.6435613172392</v>
       </c>
     </row>
     <row r="251">
@@ -2382,7 +2382,7 @@
         <v>2011-10</v>
       </c>
       <c r="B251">
-        <v>87.3590578534289</v>
+        <v>87.360847150079</v>
       </c>
     </row>
     <row r="252">
@@ -2390,7 +2390,7 @@
         <v>2011-11</v>
       </c>
       <c r="B252">
-        <v>91.3311504078716</v>
+        <v>91.332330595755</v>
       </c>
     </row>
     <row r="253">
@@ -2398,7 +2398,7 @@
         <v>2011-12</v>
       </c>
       <c r="B253">
-        <v>92.2431739826039</v>
+        <v>92.2428024826428</v>
       </c>
     </row>
     <row r="254">
@@ -2406,7 +2406,7 @@
         <v>2012-01</v>
       </c>
       <c r="B254">
-        <v>93.891016738709</v>
+        <v>93.8907217026279</v>
       </c>
     </row>
     <row r="255">
@@ -2414,7 +2414,7 @@
         <v>2012-02</v>
       </c>
       <c r="B255">
-        <v>95.8545804010102</v>
+        <v>95.852332128896</v>
       </c>
     </row>
     <row r="256">
@@ -2422,7 +2422,7 @@
         <v>2012-03</v>
       </c>
       <c r="B256">
-        <v>97.3128690403867</v>
+        <v>97.3138298964379</v>
       </c>
     </row>
     <row r="257">
@@ -2430,7 +2430,7 @@
         <v>2012-04</v>
       </c>
       <c r="B257">
-        <v>98.4111237947068</v>
+        <v>98.4071449877751</v>
       </c>
     </row>
     <row r="258">
@@ -2438,7 +2438,7 @@
         <v>2012-05</v>
       </c>
       <c r="B258">
-        <v>96.3031472346549</v>
+        <v>96.3027236763132</v>
       </c>
     </row>
     <row r="259">
@@ -2446,7 +2446,7 @@
         <v>2012-06</v>
       </c>
       <c r="B259">
-        <v>97.4776955889235</v>
+        <v>97.4730085964933</v>
       </c>
     </row>
     <row r="260">
@@ -2454,7 +2454,7 @@
         <v>2012-07</v>
       </c>
       <c r="B260">
-        <v>97.8168188958181</v>
+        <v>97.8151489264133</v>
       </c>
     </row>
     <row r="261">
@@ -2462,7 +2462,7 @@
         <v>2012-08</v>
       </c>
       <c r="B261">
-        <v>102.235872101879</v>
+        <v>102.231605573822</v>
       </c>
     </row>
     <row r="262">
@@ -2470,7 +2470,7 @@
         <v>2012-09</v>
       </c>
       <c r="B262">
-        <v>102.463117794139</v>
+        <v>102.460335585394</v>
       </c>
     </row>
     <row r="263">
@@ -2478,7 +2478,7 @@
         <v>2012-10</v>
       </c>
       <c r="B263">
-        <v>100.11057013166</v>
+        <v>100.107479358468</v>
       </c>
     </row>
     <row r="264">
@@ -2486,7 +2486,7 @@
         <v>2012-11</v>
       </c>
       <c r="B264">
-        <v>98.9100461994618</v>
+        <v>98.9070984391654</v>
       </c>
     </row>
     <row r="265">
@@ -2494,7 +2494,7 @@
         <v>2012-12</v>
       </c>
       <c r="B265">
-        <v>101.7633726569</v>
+        <v>101.762371130262</v>
       </c>
     </row>
     <row r="266">
@@ -2502,7 +2502,7 @@
         <v>2013-01</v>
       </c>
       <c r="B266">
-        <v>103.054806860923</v>
+        <v>103.052139897194</v>
       </c>
     </row>
     <row r="267">
@@ -2510,7 +2510,7 @@
         <v>2013-02</v>
       </c>
       <c r="B267">
-        <v>104.6661412622</v>
+        <v>104.663213907421</v>
       </c>
     </row>
     <row r="268">
@@ -2518,7 +2518,7 @@
         <v>2013-03</v>
       </c>
       <c r="B268">
-        <v>103.137029794214</v>
+        <v>103.135494807407</v>
       </c>
     </row>
     <row r="269">
@@ -2526,7 +2526,7 @@
         <v>2013-04</v>
       </c>
       <c r="B269">
-        <v>101.092400251639</v>
+        <v>101.093133150523</v>
       </c>
     </row>
     <row r="270">
@@ -2534,7 +2534,7 @@
         <v>2013-05</v>
       </c>
       <c r="B270">
-        <v>102.673872337516</v>
+        <v>102.671495951533</v>
       </c>
     </row>
     <row r="271">
@@ -2542,7 +2542,7 @@
         <v>2013-06</v>
       </c>
       <c r="B271">
-        <v>101.158722427788</v>
+        <v>101.161703541251</v>
       </c>
     </row>
     <row r="272">
@@ -2550,7 +2550,7 @@
         <v>2013-07</v>
       </c>
       <c r="B272">
-        <v>104.18405876007</v>
+        <v>104.181342609807</v>
       </c>
     </row>
     <row r="273">
@@ -2558,7 +2558,7 @@
         <v>2013-08</v>
       </c>
       <c r="B273">
-        <v>103.613555595679</v>
+        <v>103.613836478245</v>
       </c>
     </row>
     <row r="274">
@@ -2566,7 +2566,7 @@
         <v>2013-09</v>
       </c>
       <c r="B274">
-        <v>105.965595046092</v>
+        <v>105.966420122161</v>
       </c>
     </row>
     <row r="275">
@@ -2574,7 +2574,7 @@
         <v>2013-10</v>
       </c>
       <c r="B275">
-        <v>106.108397800495</v>
+        <v>106.108170029065</v>
       </c>
     </row>
     <row r="276">
@@ -2582,7 +2582,7 @@
         <v>2013-11</v>
       </c>
       <c r="B276">
-        <v>104.948767164286</v>
+        <v>104.946420743517</v>
       </c>
     </row>
     <row r="277">
@@ -2590,7 +2590,7 @@
         <v>2013-12</v>
       </c>
       <c r="B277">
-        <v>107.744404384271</v>
+        <v>107.746021246246</v>
       </c>
     </row>
     <row r="278">
@@ -2598,7 +2598,7 @@
         <v>2014-01</v>
       </c>
       <c r="B278">
-        <v>104.328089416024</v>
+        <v>104.327870468955</v>
       </c>
     </row>
     <row r="279">
@@ -2606,7 +2606,7 @@
         <v>2014-02</v>
       </c>
       <c r="B279">
-        <v>106.562123317043</v>
+        <v>106.563109967869</v>
       </c>
     </row>
     <row r="280">
@@ -2614,7 +2614,7 @@
         <v>2014-03</v>
       </c>
       <c r="B280">
-        <v>103.093757157434</v>
+        <v>103.092160848367</v>
       </c>
     </row>
     <row r="281">
@@ -2622,7 +2622,7 @@
         <v>2014-04</v>
       </c>
       <c r="B281">
-        <v>103.341244177062</v>
+        <v>103.340673917205</v>
       </c>
     </row>
     <row r="282">
@@ -2630,7 +2630,7 @@
         <v>2014-05</v>
       </c>
       <c r="B282">
-        <v>102.90277562023</v>
+        <v>102.90169915946</v>
       </c>
     </row>
     <row r="283">
@@ -2638,7 +2638,7 @@
         <v>2014-06</v>
       </c>
       <c r="B283">
-        <v>103.75826428724</v>
+        <v>103.757831976258</v>
       </c>
     </row>
     <row r="284">
@@ -2646,7 +2646,7 @@
         <v>2014-07</v>
       </c>
       <c r="B284">
-        <v>99.62364683147</v>
+        <v>99.6250062651144</v>
       </c>
     </row>
     <row r="285">
@@ -2654,7 +2654,7 @@
         <v>2014-08</v>
       </c>
       <c r="B285">
-        <v>100.650353716865</v>
+        <v>100.64640277052</v>
       </c>
     </row>
     <row r="286">
@@ -2662,7 +2662,7 @@
         <v>2014-09</v>
       </c>
       <c r="B286">
-        <v>98.5851561165079</v>
+        <v>98.5862458548339</v>
       </c>
     </row>
     <row r="287">
@@ -2670,7 +2670,7 @@
         <v>2014-10</v>
       </c>
       <c r="B287">
-        <v>97.4683772717542</v>
+        <v>97.4672500546251</v>
       </c>
     </row>
     <row r="288">
@@ -2678,7 +2678,7 @@
         <v>2014-11</v>
       </c>
       <c r="B288">
-        <v>96.6039073933258</v>
+        <v>96.6083060135851</v>
       </c>
     </row>
     <row r="289">
@@ -2686,7 +2686,7 @@
         <v>2014-12</v>
       </c>
       <c r="B289">
-        <v>95.3685388990883</v>
+        <v>95.3659158764221</v>
       </c>
     </row>
     <row r="290">
@@ -2694,7 +2694,7 @@
         <v>2015-01</v>
       </c>
       <c r="B290">
-        <v>94.1043887740594</v>
+        <v>94.1042253000545</v>
       </c>
     </row>
     <row r="291">
@@ -2702,7 +2702,7 @@
         <v>2015-02</v>
       </c>
       <c r="B291">
-        <v>82.6488317957572</v>
+        <v>82.6517747635004</v>
       </c>
     </row>
     <row r="292">
@@ -2710,7 +2710,7 @@
         <v>2015-03</v>
       </c>
       <c r="B292">
-        <v>89.6925274120494</v>
+        <v>89.6939506738068</v>
       </c>
     </row>
     <row r="293">
@@ -2718,7 +2718,7 @@
         <v>2015-04</v>
       </c>
       <c r="B293">
-        <v>86.8103316679221</v>
+        <v>86.8121782790229</v>
       </c>
     </row>
     <row r="294">
@@ -2726,7 +2726,7 @@
         <v>2015-05</v>
       </c>
       <c r="B294">
-        <v>93.690763438049</v>
+        <v>93.6920397220786</v>
       </c>
     </row>
     <row r="295">
@@ -2734,7 +2734,7 @@
         <v>2015-06</v>
       </c>
       <c r="B295">
-        <v>93.2196758855259</v>
+        <v>93.2203469208262</v>
       </c>
     </row>
     <row r="296">
@@ -2742,7 +2742,7 @@
         <v>2015-07</v>
       </c>
       <c r="B296">
-        <v>96.9419373912611</v>
+        <v>96.9393284402578</v>
       </c>
     </row>
     <row r="297">
@@ -2750,7 +2750,7 @@
         <v>2015-08</v>
       </c>
       <c r="B297">
-        <v>98.5956132688595</v>
+        <v>98.5982150222087</v>
       </c>
     </row>
     <row r="298">
@@ -2758,7 +2758,7 @@
         <v>2015-09</v>
       </c>
       <c r="B298">
-        <v>97.6497637373112</v>
+        <v>97.6461600136668</v>
       </c>
     </row>
     <row r="299">
@@ -2766,7 +2766,7 @@
         <v>2015-10</v>
       </c>
       <c r="B299">
-        <v>99.557940621381</v>
+        <v>99.5551828091413</v>
       </c>
     </row>
     <row r="300">
@@ -2774,7 +2774,7 @@
         <v>2015-11</v>
       </c>
       <c r="B300">
-        <v>99.7481179291834</v>
+        <v>99.7443000967261</v>
       </c>
     </row>
     <row r="301">
@@ -2782,7 +2782,7 @@
         <v>2015-12</v>
       </c>
       <c r="B301">
-        <v>97.6542565019753</v>
+        <v>97.6521916685669</v>
       </c>
     </row>
     <row r="302">
@@ -2790,7 +2790,7 @@
         <v>2016-01</v>
       </c>
       <c r="B302">
-        <v>97.8134780222407</v>
+        <v>97.8095747830868</v>
       </c>
     </row>
     <row r="303">
@@ -2798,7 +2798,7 @@
         <v>2016-02</v>
       </c>
       <c r="B303">
-        <v>101.041066620592</v>
+        <v>101.037891833731</v>
       </c>
     </row>
     <row r="304">
@@ -2806,7 +2806,7 @@
         <v>2016-03</v>
       </c>
       <c r="B304">
-        <v>98.6746632548598</v>
+        <v>98.6708470750573</v>
       </c>
     </row>
     <row r="305">
@@ -2814,7 +2814,7 @@
         <v>2016-04</v>
       </c>
       <c r="B305">
-        <v>101.883387885144</v>
+        <v>101.878150385777</v>
       </c>
     </row>
     <row r="306">
@@ -2822,7 +2822,7 @@
         <v>2016-05</v>
       </c>
       <c r="B306">
-        <v>99.274115512051</v>
+        <v>99.2699407207286</v>
       </c>
     </row>
     <row r="307">
@@ -2830,7 +2830,7 @@
         <v>2016-06</v>
       </c>
       <c r="B307">
-        <v>100.828923590076</v>
+        <v>100.825249685755</v>
       </c>
     </row>
     <row r="308">
@@ -2838,7 +2838,7 @@
         <v>2016-07</v>
       </c>
       <c r="B308">
-        <v>100.904842305208</v>
+        <v>100.901692125495</v>
       </c>
     </row>
     <row r="309">
@@ -2846,7 +2846,7 @@
         <v>2016-08</v>
       </c>
       <c r="B309">
-        <v>99.7981909280082</v>
+        <v>99.7971829472391</v>
       </c>
     </row>
     <row r="310">
@@ -2854,7 +2854,7 @@
         <v>2016-09</v>
       </c>
       <c r="B310">
-        <v>100.716245299453</v>
+        <v>100.710985777028</v>
       </c>
     </row>
     <row r="311">
@@ -2862,7 +2862,7 @@
         <v>2016-10</v>
       </c>
       <c r="B311">
-        <v>101.163278619866</v>
+        <v>101.161767704295</v>
       </c>
     </row>
     <row r="312">
@@ -2870,7 +2870,7 @@
         <v>2016-11</v>
       </c>
       <c r="B312">
-        <v>101.653114615916</v>
+        <v>101.648466933533</v>
       </c>
     </row>
     <row r="313">
@@ -2878,7 +2878,7 @@
         <v>2016-12</v>
       </c>
       <c r="B313">
-        <v>101.658598523382</v>
+        <v>101.656296810941</v>
       </c>
     </row>
     <row r="314">
@@ -2886,7 +2886,7 @@
         <v>2017-01</v>
       </c>
       <c r="B314">
-        <v>105.223190177086</v>
+        <v>105.219853680811</v>
       </c>
     </row>
     <row r="315">
@@ -2894,7 +2894,7 @@
         <v>2017-02</v>
       </c>
       <c r="B315">
-        <v>107.009545798392</v>
+        <v>107.006611748723</v>
       </c>
     </row>
     <row r="316">
@@ -2902,7 +2902,7 @@
         <v>2017-03</v>
       </c>
       <c r="B316">
-        <v>110.853042827275</v>
+        <v>110.850138424511</v>
       </c>
     </row>
     <row r="317">
@@ -2910,7 +2910,7 @@
         <v>2017-04</v>
       </c>
       <c r="B317">
-        <v>108.467405099426</v>
+        <v>108.467296746047</v>
       </c>
     </row>
     <row r="318">
@@ -2918,7 +2918,7 @@
         <v>2017-05</v>
       </c>
       <c r="B318">
-        <v>108.700222833866</v>
+        <v>108.69401956008</v>
       </c>
     </row>
     <row r="319">
@@ -2926,7 +2926,7 @@
         <v>2017-06</v>
       </c>
       <c r="B319">
-        <v>107.825448442881</v>
+        <v>107.822186639816</v>
       </c>
     </row>
     <row r="320">
@@ -2934,7 +2934,7 @@
         <v>2017-07</v>
       </c>
       <c r="B320">
-        <v>109.669697600798</v>
+        <v>109.669518180426</v>
       </c>
     </row>
     <row r="321">
@@ -2942,7 +2942,7 @@
         <v>2017-08</v>
       </c>
       <c r="B321">
-        <v>107.196953888601</v>
+        <v>107.191733233216</v>
       </c>
     </row>
     <row r="322">
@@ -2950,7 +2950,7 @@
         <v>2017-09</v>
       </c>
       <c r="B322">
-        <v>111.061902112265</v>
+        <v>111.06033752719</v>
       </c>
     </row>
     <row r="323">
@@ -2958,7 +2958,7 @@
         <v>2017-10</v>
       </c>
       <c r="B323">
-        <v>110.511903127459</v>
+        <v>110.509843596978</v>
       </c>
     </row>
     <row r="324">
@@ -2966,7 +2966,7 @@
         <v>2017-11</v>
       </c>
       <c r="B324">
-        <v>110.087460131144</v>
+        <v>110.085286334734</v>
       </c>
     </row>
     <row r="325">
@@ -2974,7 +2974,7 @@
         <v>2017-12</v>
       </c>
       <c r="B325">
-        <v>110.398309376285</v>
+        <v>110.395691366425</v>
       </c>
     </row>
     <row r="326">
@@ -2982,7 +2982,7 @@
         <v>2018-01</v>
       </c>
       <c r="B326">
-        <v>108.402238656757</v>
+        <v>108.402115011111</v>
       </c>
     </row>
     <row r="327">
@@ -2990,7 +2990,7 @@
         <v>2018-02</v>
       </c>
       <c r="B327">
-        <v>103.801720487573</v>
+        <v>103.799134969351</v>
       </c>
     </row>
     <row r="328">
@@ -2998,7 +2998,7 @@
         <v>2018-03</v>
       </c>
       <c r="B328">
-        <v>100.778083417295</v>
+        <v>100.776787294798</v>
       </c>
     </row>
     <row r="329">
@@ -3006,7 +3006,7 @@
         <v>2018-04</v>
       </c>
       <c r="B329">
-        <v>102.670177332309</v>
+        <v>102.668262417446</v>
       </c>
     </row>
     <row r="330">
@@ -3014,7 +3014,7 @@
         <v>2018-05</v>
       </c>
       <c r="B330">
-        <v>101.185015306354</v>
+        <v>101.187201300162</v>
       </c>
     </row>
     <row r="331">
@@ -3022,7 +3022,7 @@
         <v>2018-06</v>
       </c>
       <c r="B331">
-        <v>99.3970557841497</v>
+        <v>99.3938747032815</v>
       </c>
     </row>
     <row r="332">
@@ -3030,7 +3030,7 @@
         <v>2018-07</v>
       </c>
       <c r="B332">
-        <v>99.1216382165153</v>
+        <v>99.1203674354043</v>
       </c>
     </row>
     <row r="333">
@@ -3038,7 +3038,7 @@
         <v>2018-08</v>
       </c>
       <c r="B333">
-        <v>97.1101893416826</v>
+        <v>97.1093077934743</v>
       </c>
     </row>
     <row r="334">
@@ -3046,7 +3046,7 @@
         <v>2018-09</v>
       </c>
       <c r="B334">
-        <v>97.2805665098484</v>
+        <v>97.2789787219334</v>
       </c>
     </row>
     <row r="335">
@@ -3054,7 +3054,7 @@
         <v>2018-10</v>
       </c>
       <c r="B335">
-        <v>95.9552343947421</v>
+        <v>95.9531969034322</v>
       </c>
     </row>
     <row r="336">
@@ -3062,7 +3062,7 @@
         <v>2018-11</v>
       </c>
       <c r="B336">
-        <v>94.505303067643</v>
+        <v>94.5026356517619</v>
       </c>
     </row>
     <row r="337">
@@ -3070,7 +3070,7 @@
         <v>2018-12</v>
       </c>
       <c r="B337">
-        <v>94.0444453391927</v>
+        <v>94.0438815631617</v>
       </c>
     </row>
     <row r="338">
@@ -3078,7 +3078,7 @@
         <v>2019-01</v>
       </c>
       <c r="B338">
-        <v>93.5910312487052</v>
+        <v>93.5882229956796</v>
       </c>
     </row>
     <row r="339">
@@ -3086,7 +3086,7 @@
         <v>2019-02</v>
       </c>
       <c r="B339">
-        <v>95.2124443675203</v>
+        <v>95.208521433469</v>
       </c>
     </row>
     <row r="340">
@@ -3094,7 +3094,7 @@
         <v>2019-03</v>
       </c>
       <c r="B340">
-        <v>96.7033462973756</v>
+        <v>96.6997813071399</v>
       </c>
     </row>
     <row r="341">
@@ -3102,7 +3102,7 @@
         <v>2019-04</v>
       </c>
       <c r="B341">
-        <v>95.7739390220707</v>
+        <v>95.773273780937</v>
       </c>
     </row>
     <row r="342">
@@ -3110,7 +3110,7 @@
         <v>2019-05</v>
       </c>
       <c r="B342">
-        <v>95.0894891305442</v>
+        <v>95.0825769227885</v>
       </c>
     </row>
     <row r="343">
@@ -3118,7 +3118,7 @@
         <v>2019-06</v>
       </c>
       <c r="B343">
-        <v>94.8406475246689</v>
+        <v>94.8393857437687</v>
       </c>
     </row>
     <row r="344">
@@ -3126,7 +3126,7 @@
         <v>2019-07</v>
       </c>
       <c r="B344">
-        <v>93.3143868636081</v>
+        <v>93.312249364206</v>
       </c>
     </row>
     <row r="345">
@@ -3134,7 +3134,7 @@
         <v>2019-08</v>
       </c>
       <c r="B345">
-        <v>95.0004700315778</v>
+        <v>94.9953671393737</v>
       </c>
     </row>
     <row r="346">
@@ -3142,7 +3142,7 @@
         <v>2019-09</v>
       </c>
       <c r="B346">
-        <v>95.2315583104494</v>
+        <v>95.2288721616925</v>
       </c>
     </row>
     <row r="347">
@@ -3150,7 +3150,7 @@
         <v>2019-10</v>
       </c>
       <c r="B347">
-        <v>94.0058563332153</v>
+        <v>94.0041365054506</v>
       </c>
     </row>
     <row r="348">
@@ -3158,7 +3158,7 @@
         <v>2019-11</v>
       </c>
       <c r="B348">
-        <v>97.2597744416025</v>
+        <v>97.2531497029417</v>
       </c>
     </row>
     <row r="349">
@@ -3166,7 +3166,7 @@
         <v>2019-12</v>
       </c>
       <c r="B349">
-        <v>99.0052099593167</v>
+        <v>99.0022006101416</v>
       </c>
     </row>
     <row r="350">
@@ -3174,7 +3174,7 @@
         <v>2020-01</v>
       </c>
       <c r="B350">
-        <v>101.532904968387</v>
+        <v>101.530957075245</v>
       </c>
     </row>
     <row r="351">
@@ -3182,7 +3182,7 @@
         <v>2020-02</v>
       </c>
       <c r="B351">
-        <v>96.1163529977255</v>
+        <v>96.1083757034354</v>
       </c>
     </row>
     <row r="352">
@@ -3190,7 +3190,7 @@
         <v>2020-03</v>
       </c>
       <c r="B352">
-        <v>81.6347584112973</v>
+        <v>81.6202133089814</v>
       </c>
     </row>
     <row r="353">
@@ -3198,7 +3198,7 @@
         <v>2020-04</v>
       </c>
       <c r="B353">
-        <v>57.0639921039906</v>
+        <v>57.0546396208403</v>
       </c>
     </row>
     <row r="354">
@@ -3206,7 +3206,7 @@
         <v>2020-05</v>
       </c>
       <c r="B354">
-        <v>69.3062846871514</v>
+        <v>69.2949237018685</v>
       </c>
     </row>
     <row r="355">
@@ -3214,7 +3214,7 @@
         <v>2020-06</v>
       </c>
       <c r="B355">
-        <v>101.148222681674</v>
+        <v>101.139061996805</v>
       </c>
     </row>
     <row r="356">
@@ -3222,7 +3222,7 @@
         <v>2020-07</v>
       </c>
       <c r="B356">
-        <v>118.50188953483</v>
+        <v>118.495664152051</v>
       </c>
     </row>
     <row r="357">
@@ -3230,7 +3230,7 @@
         <v>2020-08</v>
       </c>
       <c r="B357">
-        <v>119.860265232463</v>
+        <v>119.856984383058</v>
       </c>
     </row>
     <row r="358">
@@ -3238,7 +3238,7 @@
         <v>2020-09</v>
       </c>
       <c r="B358">
-        <v>113.826865273309</v>
+        <v>113.82242239916</v>
       </c>
     </row>
     <row r="359">
@@ -3246,7 +3246,7 @@
         <v>2020-10</v>
       </c>
       <c r="B359">
-        <v>115.000790385203</v>
+        <v>114.998046997073</v>
       </c>
     </row>
     <row r="360">
@@ -3254,7 +3254,7 @@
         <v>2020-11</v>
       </c>
       <c r="B360">
-        <v>106.469599408022</v>
+        <v>106.469137695248</v>
       </c>
     </row>
     <row r="361">
@@ -3262,7 +3262,7 @@
         <v>2020-12</v>
       </c>
       <c r="B361">
-        <v>109.652621646243</v>
+        <v>109.654717101879</v>
       </c>
     </row>
     <row r="362">
@@ -3270,7 +3270,7 @@
         <v>2021-01</v>
       </c>
       <c r="B362">
-        <v>106.723972490371</v>
+        <v>106.722243996046</v>
       </c>
     </row>
     <row r="363">
@@ -3278,7 +3278,7 @@
         <v>2021-02</v>
       </c>
       <c r="B363">
-        <v>116.052494969314</v>
+        <v>116.052643121571</v>
       </c>
     </row>
     <row r="364">
@@ -3286,7 +3286,7 @@
         <v>2021-03</v>
       </c>
       <c r="B364">
-        <v>120.787003911084</v>
+        <v>120.782118943097</v>
       </c>
     </row>
     <row r="365">
@@ -3294,7 +3294,7 @@
         <v>2021-04</v>
       </c>
       <c r="B365">
-        <v>129.491556835723</v>
+        <v>129.487650779598</v>
       </c>
     </row>
     <row r="366">
@@ -3302,7 +3302,7 @@
         <v>2021-05</v>
       </c>
       <c r="B366">
-        <v>126.755506987557</v>
+        <v>126.754114313183</v>
       </c>
     </row>
     <row r="367">
@@ -3310,7 +3310,7 @@
         <v>2021-06</v>
       </c>
       <c r="B367">
-        <v>116.33185687586</v>
+        <v>116.329833943175</v>
       </c>
     </row>
     <row r="368">
@@ -3318,7 +3318,7 @@
         <v>2021-07</v>
       </c>
       <c r="B368">
-        <v>121.703019558735</v>
+        <v>121.697548918849</v>
       </c>
     </row>
     <row r="369">
@@ -3326,7 +3326,7 @@
         <v>2021-08</v>
       </c>
       <c r="B369">
-        <v>112.155676408285</v>
+        <v>112.153058304825</v>
       </c>
     </row>
     <row r="370">
@@ -3334,7 +3334,7 @@
         <v>2021-09</v>
       </c>
       <c r="B370">
-        <v>110.748117656858</v>
+        <v>110.742909178583</v>
       </c>
     </row>
     <row r="371">
@@ -3342,7 +3342,7 @@
         <v>2021-10</v>
       </c>
       <c r="B371">
-        <v>108.339593059584</v>
+        <v>108.336075924385</v>
       </c>
     </row>
     <row r="372">
@@ -3350,7 +3350,7 @@
         <v>2021-11</v>
       </c>
       <c r="B372">
-        <v>107.460387787913</v>
+        <v>107.455924672638</v>
       </c>
     </row>
     <row r="373">
@@ -3358,7 +3358,7 @@
         <v>2021-12</v>
       </c>
       <c r="B373">
-        <v>103.546399874564</v>
+        <v>103.538266183185</v>
       </c>
     </row>
     <row r="374">
@@ -3366,7 +3366,7 @@
         <v>2022-01</v>
       </c>
       <c r="B374">
-        <v>102.646846395563</v>
+        <v>102.647016690337</v>
       </c>
     </row>
     <row r="375">
@@ -3374,7 +3374,7 @@
         <v>2022-02</v>
       </c>
       <c r="B375">
-        <v>101.571062532119</v>
+        <v>101.563855996434</v>
       </c>
     </row>
     <row r="376">
@@ -3382,7 +3382,7 @@
         <v>2022-03</v>
       </c>
       <c r="B376">
-        <v>96.6690922159084</v>
+        <v>96.661904982514</v>
       </c>
     </row>
     <row r="377">
@@ -3390,7 +3390,7 @@
         <v>2022-04</v>
       </c>
       <c r="B377">
-        <v>96.6927009049553</v>
+        <v>96.688957799676</v>
       </c>
     </row>
     <row r="378">
@@ -3398,7 +3398,7 @@
         <v>2022-05</v>
       </c>
       <c r="B378">
-        <v>91.0710705259633</v>
+        <v>91.0705828089144</v>
       </c>
     </row>
     <row r="379">
@@ -3406,7 +3406,7 @@
         <v>2022-06</v>
       </c>
       <c r="B379">
-        <v>92.6685879345387</v>
+        <v>92.6662864447899</v>
       </c>
     </row>
     <row r="380">
@@ -3414,7 +3414,7 @@
         <v>2022-07</v>
       </c>
       <c r="B380">
-        <v>89.3933120541148</v>
+        <v>89.3946736130477</v>
       </c>
     </row>
     <row r="381">
@@ -3422,7 +3422,7 @@
         <v>2022-08</v>
       </c>
       <c r="B381">
-        <v>86.6880299098844</v>
+        <v>86.6888944237162</v>
       </c>
     </row>
     <row r="382">
@@ -3430,7 +3430,7 @@
         <v>2022-09</v>
       </c>
       <c r="B382">
-        <v>86.2653668702287</v>
+        <v>86.2638596951111</v>
       </c>
     </row>
     <row r="383">
@@ -3438,7 +3438,7 @@
         <v>2022-10</v>
       </c>
       <c r="B383">
-        <v>87.750779263138</v>
+        <v>87.7507133967727</v>
       </c>
     </row>
     <row r="384">
@@ -3446,7 +3446,7 @@
         <v>2022-11</v>
       </c>
       <c r="B384">
-        <v>89.3369419847469</v>
+        <v>89.3311813252431</v>
       </c>
     </row>
     <row r="385">
@@ -3454,7 +3454,7 @@
         <v>2022-12</v>
       </c>
       <c r="B385">
-        <v>89.3027615395066</v>
+        <v>89.3020371184045</v>
       </c>
     </row>
     <row r="386">
@@ -3462,7 +3462,7 @@
         <v>2023-01</v>
       </c>
       <c r="B386">
-        <v>92.2230421497889</v>
+        <v>92.2242430100584</v>
       </c>
     </row>
     <row r="387">
@@ -3470,7 +3470,7 @@
         <v>2023-02</v>
       </c>
       <c r="B387">
-        <v>91.1340193526542</v>
+        <v>91.1342608900201</v>
       </c>
     </row>
     <row r="388">
@@ -3478,7 +3478,7 @@
         <v>2023-03</v>
       </c>
       <c r="B388">
-        <v>96.0205047678048</v>
+        <v>96.021324535786</v>
       </c>
     </row>
     <row r="389">
@@ -3486,7 +3486,7 @@
         <v>2023-04</v>
       </c>
       <c r="B389">
-        <v>91.5281847813641</v>
+        <v>91.5322446077977</v>
       </c>
     </row>
     <row r="390">
@@ -3494,7 +3494,7 @@
         <v>2023-05</v>
       </c>
       <c r="B390">
-        <v>90.9347219912685</v>
+        <v>90.9412867379826</v>
       </c>
     </row>
     <row r="391">
@@ -3502,7 +3502,7 @@
         <v>2023-06</v>
       </c>
       <c r="B391">
-        <v>89.8316031201805</v>
+        <v>89.841348173302</v>
       </c>
     </row>
     <row r="392">
@@ -3510,7 +3510,7 @@
         <v>2023-07</v>
       </c>
       <c r="B392">
-        <v>88.9718333792136</v>
+        <v>88.979853313258</v>
       </c>
     </row>
     <row r="393">
@@ -3518,7 +3518,7 @@
         <v>2023-08</v>
       </c>
       <c r="B393">
-        <v>90.9096299561668</v>
+        <v>90.9192557019232</v>
       </c>
     </row>
     <row r="394">
@@ -3526,7 +3526,7 @@
         <v>2023-09</v>
       </c>
       <c r="B394">
-        <v>95.301443305813</v>
+        <v>95.3122049176482</v>
       </c>
     </row>
     <row r="395">
@@ -3534,7 +3534,7 @@
         <v>2023-10</v>
       </c>
       <c r="B395">
-        <v>94.419902031799</v>
+        <v>94.4253548655085</v>
       </c>
     </row>
     <row r="396">
@@ -3542,7 +3542,7 @@
         <v>2023-11</v>
       </c>
       <c r="B396">
-        <v>98.7151010259861</v>
+        <v>98.7232950053536</v>
       </c>
     </row>
     <row r="397">
@@ -3550,7 +3550,7 @@
         <v>2023-12</v>
       </c>
       <c r="B397">
-        <v>101.602092975742</v>
+        <v>101.610739201483</v>
       </c>
     </row>
     <row r="398">
@@ -3558,7 +3558,7 @@
         <v>2024-01</v>
       </c>
       <c r="B398">
-        <v>96.9973478955211</v>
+        <v>97.0087783089715</v>
       </c>
     </row>
     <row r="399">
@@ -3566,7 +3566,7 @@
         <v>2024-02</v>
       </c>
       <c r="B399">
-        <v>99.2805541156273</v>
+        <v>99.2897761532804</v>
       </c>
     </row>
     <row r="400">
@@ -3574,7 +3574,7 @@
         <v>2024-03</v>
       </c>
       <c r="B400">
-        <v>98.9938990866041</v>
+        <v>99.0048699428032</v>
       </c>
     </row>
     <row r="401">
@@ -3582,7 +3582,7 @@
         <v>2024-04</v>
       </c>
       <c r="B401">
-        <v>102.283435870214</v>
+        <v>102.293041908695</v>
       </c>
     </row>
     <row r="402">
@@ -3590,7 +3590,7 @@
         <v>2024-05</v>
       </c>
       <c r="B402">
-        <v>104.835128647315</v>
+        <v>104.851365510365</v>
       </c>
     </row>
     <row r="403">
@@ -3598,7 +3598,7 @@
         <v>2024-06</v>
       </c>
       <c r="B403">
-        <v>104.39802669217</v>
+        <v>104.419754735234</v>
       </c>
     </row>
     <row r="404">
@@ -3606,7 +3606,7 @@
         <v>2024-07</v>
       </c>
       <c r="B404">
-        <v>101.960724496266</v>
+        <v>101.970449317908</v>
       </c>
     </row>
     <row r="405">
@@ -3614,7 +3614,7 @@
         <v>2024-08</v>
       </c>
       <c r="B405">
-        <v>105.260260355858</v>
+        <v>105.284949571959</v>
       </c>
     </row>
     <row r="406">
@@ -3622,7 +3622,7 @@
         <v>2024-09</v>
       </c>
       <c r="B406">
-        <v>103.690021230526</v>
+        <v>103.715425392086</v>
       </c>
     </row>
     <row r="407">
@@ -3630,7 +3630,7 @@
         <v>2024-10</v>
       </c>
       <c r="B407">
-        <v>100.286888975034</v>
+        <v>100.301706250181</v>
       </c>
     </row>
     <row r="408">
@@ -3638,7 +3638,7 @@
         <v>2024-11</v>
       </c>
       <c r="B408">
-        <v>98.4478458007607</v>
+        <v>98.4669097693332</v>
       </c>
     </row>
     <row r="409">
@@ -3646,7 +3646,7 @@
         <v>2024-12</v>
       </c>
       <c r="B409">
-        <v>99.6981457191873</v>
+        <v>99.7261265049334</v>
       </c>
     </row>
     <row r="410">
@@ -3654,7 +3654,7 @@
         <v>2025-01</v>
       </c>
       <c r="B410">
-        <v>102.803247773728</v>
+        <v>102.824482016473</v>
       </c>
     </row>
     <row r="411">
@@ -3662,7 +3662,7 @@
         <v>2025-02</v>
       </c>
       <c r="B411">
-        <v>102.861452984304</v>
+        <v>102.84901544212</v>
       </c>
     </row>
     <row r="412">
@@ -3670,7 +3670,7 @@
         <v>2025-03</v>
       </c>
       <c r="B412">
-        <v>100.867818053387</v>
+        <v>100.909796999939</v>
       </c>
     </row>
     <row r="413">
@@ -3678,7 +3678,7 @@
         <v>2025-04</v>
       </c>
       <c r="B413">
-        <v>95.3376673713961</v>
+        <v>95.3741683630073</v>
       </c>
     </row>
     <row r="414">
@@ -3686,7 +3686,7 @@
         <v>2025-05</v>
       </c>
       <c r="B414">
-        <v>97.622435790928</v>
+        <v>97.6584445407097</v>
       </c>
     </row>
     <row r="415">
@@ -3694,7 +3694,7 @@
         <v>2025-06</v>
       </c>
       <c r="B415">
-        <v>95.4311215778749</v>
+        <v>95.4901612460777</v>
       </c>
     </row>
     <row r="416">
@@ -3702,7 +3702,7 @@
         <v>2025-07</v>
       </c>
       <c r="B416">
-        <v>100.844386403688</v>
+        <v>100.854128592472</v>
       </c>
     </row>
     <row r="417">
@@ -3710,7 +3710,7 @@
         <v>2025-08</v>
       </c>
       <c r="B417">
-        <v>97.3031587253431</v>
+        <v>97.3414284752353</v>
       </c>
     </row>
     <row r="418">
@@ -3718,7 +3718,7 @@
         <v>2025-09</v>
       </c>
       <c r="B418">
-        <v>97.9388858359525</v>
+        <v>97.8863254473197</v>
       </c>
     </row>
     <row r="419">
@@ -3726,7 +3726,7 @@
         <v>2025-10</v>
       </c>
       <c r="B419">
-        <v>101.385201262445</v>
+        <v>101.394905274709</v>
       </c>
     </row>
     <row r="420">
@@ -3734,7 +3734,7 @@
         <v>2025-11</v>
       </c>
       <c r="B420">
-        <v>101.550040811305</v>
+        <v>101.558225453391</v>
       </c>
     </row>
     <row r="421">
@@ -3742,7 +3742,7 @@
         <v>2025-12</v>
       </c>
       <c r="B421">
-        <v>103.641944894089</v>
+        <v>103.657188732382</v>
       </c>
     </row>
     <row r="422">
@@ -3750,7 +3750,7 @@
         <v>2026-01</v>
       </c>
       <c r="B422">
-        <v>103.324581555282</v>
+        <v>103.34745138697</v>
       </c>
     </row>
     <row r="423">
@@ -3758,7 +3758,7 @@
         <v>2026-02</v>
       </c>
       <c r="B423">
-        <v>103.795526276926</v>
+        <v>103.776058293403</v>
       </c>
     </row>
     <row r="424">
@@ -3766,12 +3766,20 @@
         <v>2026-03</v>
       </c>
       <c r="B424">
-        <v>96.1224511710867</v>
+        <v>95.6228734317395</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>2026-04</v>
+      </c>
+      <c r="B425">
+        <v>97.9266270931402</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B424"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B425"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>